<commit_message>
Corregir 3 cantidades de salsa golf y base yasaytame registradas como kilos (son gramos)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VB7LeCNjmE5MU9i5FriKqr
</commit_message>
<xml_diff>
--- a/RECETAS_CARTA_Y_POSTRES_GRAMOS.xlsx
+++ b/RECETAS_CARTA_Y_POSTRES_GRAMOS.xlsx
@@ -47,7 +47,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -79,6 +79,11 @@
         <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -107,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -120,6 +125,7 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -204,7 +210,7 @@
   <commentList>
     <comment ref="H188" authorId="0" shapeId="0">
       <text>
-        <t>Cantidad sospechosa: ya venía así en el Excel original (en kilos). Revisar.</t>
+        <t>Corregido: en Odoo decía 20 KILOS; según el costo en Inforest son 20 gramos.</t>
       </text>
     </comment>
   </commentList>
@@ -6245,8 +6251,8 @@
           <t>RB SALSA GOLF</t>
         </is>
       </c>
-      <c r="H188" s="9" t="n">
-        <v>20000</v>
+      <c r="H188" s="10" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="189">

</xml_diff>